<commit_message>
Update 2025 Annual Report on Drug-Related Mortality by revising author information, renaming the demographics chapter to data, and enhancing citations for clarity. Key changes include: - Simplified author attribution to reflect collaboration among health departments. - Renamed the chapter from "Demographics" to "Data" for better alignment with content. - Improved citation formatting in the current substance use disorder chapter for better accessibility. - Removed the demographics chapter file to streamline the report structure.
</commit_message>
<xml_diff>
--- a/data/raw/workbook.xlsx
+++ b/data/raw/workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Work Drive/GitHub/2025 Annual Report on Drug Related Mortality/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6E6657-6A2B-844B-8EC3-443AB45D1DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC88794-F1E0-264E-A188-EA72C858A792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -861,6 +861,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -895,21 +914,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="9" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -921,10 +925,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1453,7 +1453,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="E11" s="38" t="s">
+      <c r="E11" s="22" t="s">
         <v>152</v>
       </c>
       <c r="F11" t="s">
@@ -1493,22 +1493,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -1556,11 +1556,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="F5" s="16" t="s">
@@ -1580,7 +1580,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6" s="9" t="s">
         <v>116</v>
       </c>
@@ -1599,7 +1599,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7" s="9" t="s">
         <v>116</v>
       </c>
@@ -1618,7 +1618,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="F8" s="9" t="s">
         <v>116</v>
       </c>
@@ -1637,11 +1637,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9" s="9" t="s">
         <v>116</v>
       </c>
@@ -1666,7 +1666,7 @@
       <c r="B10" t="s">
         <v>120</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="F10" s="9" t="s">
         <v>119</v>
       </c>
@@ -1681,7 +1681,7 @@
       <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="F11" s="9" t="s">
         <v>119</v>
       </c>
@@ -1702,7 +1702,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="9" t="s">
         <v>118</v>
       </c>
@@ -1721,7 +1721,7 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
       <c r="F13" s="9" t="s">
         <v>118</v>
       </c>
@@ -1736,7 +1736,7 @@
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
       <c r="F14" s="9" t="s">
         <v>118</v>
       </c>
@@ -1754,7 +1754,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -1763,17 +1763,17 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -1782,20 +1782,20 @@
       <c r="B19" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -1804,25 +1804,25 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -1831,139 +1831,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2026,22 +2026,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2093,11 +2093,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="G5">
@@ -2120,7 +2120,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6" t="s">
         <v>121</v>
       </c>
@@ -2143,7 +2143,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7" t="s">
         <v>122</v>
       </c>
@@ -2166,7 +2166,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="F8" t="s">
         <v>123</v>
       </c>
@@ -2189,11 +2189,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9" t="s">
         <v>124</v>
       </c>
@@ -2222,14 +2222,14 @@
       <c r="B10" t="s">
         <v>125</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -2243,7 +2243,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -2256,13 +2256,13 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -2271,7 +2271,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -2280,17 +2280,17 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -2299,20 +2299,20 @@
       <c r="B19" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -2321,22 +2321,22 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -2345,139 +2345,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2540,22 +2540,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>152</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2607,24 +2607,24 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="34" t="s">
+      <c r="F5" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="G5" s="36">
+      <c r="G5" s="38">
         <v>2025</v>
       </c>
-      <c r="H5" s="37"/>
-      <c r="I5" s="36">
+      <c r="H5" s="39"/>
+      <c r="I5" s="38">
         <v>2024</v>
       </c>
-      <c r="J5" s="37"/>
+      <c r="J5" s="39"/>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -2633,18 +2633,18 @@
       <c r="B6" t="b">
         <v>1</v>
       </c>
-      <c r="E6" s="18"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="30" t="s">
+      <c r="E6" s="25"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="I6" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="J6" s="30" t="s">
+      <c r="J6" s="18" t="s">
         <v>17</v>
       </c>
       <c r="K6" s="2"/>
@@ -2654,20 +2654,20 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E7" s="18"/>
-      <c r="F7" s="31" t="s">
+      <c r="E7" s="25"/>
+      <c r="F7" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="20">
         <v>40</v>
       </c>
-      <c r="H7" s="33">
+      <c r="H7" s="21">
         <v>0.59699999999999998</v>
       </c>
-      <c r="I7" s="32">
+      <c r="I7" s="20">
         <v>41</v>
       </c>
-      <c r="J7" s="33">
+      <c r="J7" s="21">
         <v>0.52600000000000002</v>
       </c>
       <c r="K7" s="2"/>
@@ -2677,20 +2677,20 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E8" s="18"/>
-      <c r="F8" s="31" t="s">
+      <c r="E8" s="25"/>
+      <c r="F8" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="G8" s="32">
+      <c r="G8" s="20">
         <v>36</v>
       </c>
-      <c r="H8" s="33">
+      <c r="H8" s="21">
         <v>0.53700000000000003</v>
       </c>
-      <c r="I8" s="32">
+      <c r="I8" s="20">
         <v>46</v>
       </c>
-      <c r="J8" s="33">
+      <c r="J8" s="21">
         <v>0.59</v>
       </c>
       <c r="K8" s="2"/>
@@ -2700,24 +2700,24 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="31" t="s">
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="20">
         <v>14</v>
       </c>
-      <c r="H9" s="33">
+      <c r="H9" s="21">
         <v>0.20899999999999999</v>
       </c>
-      <c r="I9" s="32">
+      <c r="I9" s="20">
         <v>13</v>
       </c>
-      <c r="J9" s="33">
+      <c r="J9" s="21">
         <v>0.16700000000000001</v>
       </c>
       <c r="K9" s="2"/>
@@ -2730,20 +2730,20 @@
       <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="18"/>
-      <c r="F10" s="31" t="s">
+      <c r="E10" s="25"/>
+      <c r="F10" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="G10" s="32">
+      <c r="G10" s="20">
         <v>8</v>
       </c>
-      <c r="H10" s="33">
+      <c r="H10" s="21">
         <v>0.11899999999999999</v>
       </c>
-      <c r="I10" s="32">
+      <c r="I10" s="20">
         <v>5</v>
       </c>
-      <c r="J10" s="33">
+      <c r="J10" s="21">
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
@@ -2751,20 +2751,20 @@
       <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="18"/>
-      <c r="F11" s="31" t="s">
+      <c r="E11" s="25"/>
+      <c r="F11" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="G11" s="32">
+      <c r="G11" s="20">
         <v>7</v>
       </c>
-      <c r="H11" s="33">
+      <c r="H11" s="21">
         <v>0.104</v>
       </c>
-      <c r="I11" s="32">
+      <c r="I11" s="20">
         <v>4</v>
       </c>
-      <c r="J11" s="33">
+      <c r="J11" s="21">
         <v>5.0999999999999997E-2</v>
       </c>
       <c r="K11" s="1"/>
@@ -2776,20 +2776,20 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="31" t="s">
+      <c r="E12" s="25"/>
+      <c r="F12" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="G12" s="32">
+      <c r="G12" s="20">
         <v>5</v>
       </c>
-      <c r="H12" s="33">
+      <c r="H12" s="21">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="I12" s="32">
+      <c r="I12" s="20">
         <v>1</v>
       </c>
-      <c r="J12" s="33">
+      <c r="J12" s="21">
         <v>1.2999999999999999E-2</v>
       </c>
       <c r="K12" s="2"/>
@@ -2799,20 +2799,20 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
-      <c r="F13" s="31" t="s">
+      <c r="E13" s="25"/>
+      <c r="F13" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="20">
         <v>5</v>
       </c>
-      <c r="H13" s="33">
+      <c r="H13" s="21">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="I13" s="32">
+      <c r="I13" s="20">
         <v>12</v>
       </c>
-      <c r="J13" s="33">
+      <c r="J13" s="21">
         <v>0.154</v>
       </c>
     </row>
@@ -2820,20 +2820,20 @@
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
-      <c r="F14" s="31" t="s">
+      <c r="E14" s="25"/>
+      <c r="F14" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="20">
         <v>4</v>
       </c>
-      <c r="H14" s="33">
+      <c r="H14" s="21">
         <v>0.06</v>
       </c>
-      <c r="I14" s="32">
+      <c r="I14" s="20">
         <v>10</v>
       </c>
-      <c r="J14" s="33">
+      <c r="J14" s="21">
         <v>0.128</v>
       </c>
     </row>
@@ -2841,20 +2841,20 @@
       <c r="A15" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="31" t="s">
+      <c r="E15" s="25"/>
+      <c r="F15" s="19" t="s">
         <v>150</v>
       </c>
-      <c r="G15" s="32">
+      <c r="G15" s="20">
         <v>4</v>
       </c>
-      <c r="H15" s="33">
+      <c r="H15" s="21">
         <v>0.06</v>
       </c>
-      <c r="I15" s="32">
+      <c r="I15" s="20">
         <v>4</v>
       </c>
-      <c r="J15" s="33">
+      <c r="J15" s="21">
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
@@ -2862,54 +2862,54 @@
       <c r="A16" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="18"/>
-      <c r="F16" s="31" t="s">
+      <c r="E16" s="25"/>
+      <c r="F16" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="G16" s="32">
+      <c r="G16" s="20">
         <v>4</v>
       </c>
-      <c r="H16" s="33">
+      <c r="H16" s="21">
         <v>0.06</v>
       </c>
-      <c r="I16" s="32">
+      <c r="I16" s="20">
         <v>6</v>
       </c>
-      <c r="J16" s="33">
+      <c r="J16" s="21">
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="16" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -2918,25 +2918,25 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="39" t="s">
+      <c r="B22" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -2945,139 +2945,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -3152,20 +3152,20 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -3231,11 +3231,11 @@
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3246,7 +3246,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -3258,7 +3258,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -3270,7 +3270,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -3282,11 +3282,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -3304,7 +3304,7 @@
       <c r="B10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -3314,7 +3314,7 @@
       <c r="B11" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -3328,7 +3328,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -3341,13 +3341,13 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -3356,7 +3356,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -3365,36 +3365,36 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -3403,22 +3403,22 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -3427,139 +3427,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3736,23 +3736,23 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="str">
+      <c r="B1" s="24" t="str">
         <f>Master!E2</f>
         <v>Suspected Overdoses by Zip Code, 2024 vs. 2025</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -3800,11 +3800,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="F5" t="s">
@@ -3824,7 +3824,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6" t="s">
         <v>58</v>
       </c>
@@ -3843,7 +3843,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7" t="s">
         <v>59</v>
       </c>
@@ -3862,7 +3862,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="F8" t="s">
         <v>60</v>
       </c>
@@ -3881,11 +3881,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9" t="s">
         <v>61</v>
       </c>
@@ -3910,7 +3910,7 @@
       <c r="B10" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="F10" t="s">
         <v>62</v>
       </c>
@@ -3926,9 +3926,9 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11" s="18"/>
+        <v>82</v>
+      </c>
+      <c r="E11" s="25"/>
       <c r="F11" t="s">
         <v>63</v>
       </c>
@@ -3949,7 +3949,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3" t="s">
         <v>64</v>
       </c>
@@ -3968,7 +3968,7 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
       <c r="F13" t="s">
         <v>65</v>
       </c>
@@ -3983,7 +3983,7 @@
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
       <c r="F14" t="s">
         <v>66</v>
       </c>
@@ -4001,7 +4001,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
       <c r="F15" t="s">
         <v>67</v>
       </c>
@@ -4019,17 +4019,17 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -4038,20 +4038,20 @@
       <c r="B19" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -4060,22 +4060,22 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -4084,139 +4084,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -4267,22 +4267,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -4328,11 +4328,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="F5" t="s">
@@ -4349,7 +4349,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6">
         <v>2021</v>
       </c>
@@ -4366,7 +4366,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7">
         <v>2022</v>
       </c>
@@ -4383,7 +4383,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="F8">
         <v>2023</v>
       </c>
@@ -4400,11 +4400,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9">
         <v>2024</v>
       </c>
@@ -4427,7 +4427,7 @@
       <c r="B10" t="s">
         <v>80</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -4437,7 +4437,7 @@
       <c r="B11" t="s">
         <v>81</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -4451,7 +4451,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -4464,13 +4464,13 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -4479,7 +4479,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -4488,36 +4488,36 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -4526,22 +4526,22 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -4550,139 +4550,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -4745,22 +4745,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -4812,11 +4812,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="F5" t="s">
@@ -4842,7 +4842,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6">
         <v>2021</v>
       </c>
@@ -4865,7 +4865,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7">
         <v>2022</v>
       </c>
@@ -4888,7 +4888,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="F8">
         <v>2023</v>
       </c>
@@ -4911,11 +4911,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9">
         <v>2024</v>
       </c>
@@ -4944,7 +4944,7 @@
       <c r="B10" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -4954,7 +4954,7 @@
       <c r="B11" t="s">
         <v>81</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -4968,7 +4968,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -4981,13 +4981,13 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -4996,7 +4996,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -5005,17 +5005,17 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -5024,20 +5024,20 @@
       <c r="B19" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -5046,22 +5046,22 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -5070,139 +5070,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5265,22 +5265,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -5332,11 +5332,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="G5">
@@ -5359,7 +5359,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6" t="s">
         <v>88</v>
       </c>
@@ -5382,7 +5382,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -5394,7 +5394,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -5406,11 +5406,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -5428,7 +5428,7 @@
       <c r="B10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -5438,7 +5438,7 @@
       <c r="B11" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -5452,7 +5452,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -5465,13 +5465,13 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -5480,7 +5480,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -5489,17 +5489,17 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -5508,20 +5508,20 @@
       <c r="B19" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -5530,22 +5530,22 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -5554,139 +5554,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5749,22 +5749,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -5816,11 +5816,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="F5" t="s">
@@ -5846,7 +5846,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6" t="s">
         <v>90</v>
       </c>
@@ -5869,7 +5869,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7" t="s">
         <v>91</v>
       </c>
@@ -5892,7 +5892,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -5904,11 +5904,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -5926,7 +5926,7 @@
       <c r="B10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -5936,7 +5936,7 @@
       <c r="B11" t="s">
         <v>81</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -5950,7 +5950,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -5963,7 +5963,7 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -5972,7 +5972,7 @@
       <c r="B14" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -5981,7 +5981,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -5990,17 +5990,17 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -6009,20 +6009,20 @@
       <c r="B19" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -6034,22 +6034,22 @@
       <c r="B22" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -6058,139 +6058,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -6253,22 +6253,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -6320,11 +6320,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
       <c r="F5" t="s">
@@ -6350,7 +6350,7 @@
       <c r="B6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="25"/>
       <c r="F6" t="s">
         <v>95</v>
       </c>
@@ -6373,7 +6373,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7" t="s">
         <v>96</v>
       </c>
@@ -6396,7 +6396,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="F8" t="s">
         <v>97</v>
       </c>
@@ -6419,11 +6419,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9" t="s">
         <v>98</v>
       </c>
@@ -6452,7 +6452,7 @@
       <c r="B10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -6462,7 +6462,7 @@
       <c r="B11" t="s">
         <v>81</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -6476,7 +6476,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -6489,7 +6489,7 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -6498,7 +6498,7 @@
       <c r="B14" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -6507,7 +6507,7 @@
       <c r="B15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -6516,17 +6516,17 @@
       <c r="B16" t="b">
         <v>1</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -6535,20 +6535,20 @@
       <c r="B19" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -6560,22 +6560,22 @@
       <c r="B22" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -6584,139 +6584,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -6779,22 +6779,22 @@
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -6848,25 +6848,25 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="E5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="G5" s="24" t="s">
+      <c r="G5" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="H5" s="25"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="27" t="s">
+      <c r="H5" s="32"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="K5" s="28"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -6875,8 +6875,8 @@
       <c r="B6" t="b">
         <v>1</v>
       </c>
-      <c r="E6" s="18"/>
-      <c r="F6" s="23"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="30"/>
       <c r="G6" s="10">
         <v>2022</v>
       </c>
@@ -6898,7 +6898,7 @@
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E7" s="18"/>
+      <c r="E7" s="25"/>
       <c r="F7" s="12" t="s">
         <v>105</v>
       </c>
@@ -6923,7 +6923,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E8" s="18"/>
+      <c r="E8" s="25"/>
       <c r="F8" s="12" t="s">
         <v>106</v>
       </c>
@@ -6948,11 +6948,11 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="B9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9" s="12" t="s">
         <v>107</v>
       </c>
@@ -6980,7 +6980,7 @@
       <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="25"/>
       <c r="F10" s="12" t="s">
         <v>108</v>
       </c>
@@ -7004,7 +7004,7 @@
       <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="25"/>
       <c r="F11" s="12" t="s">
         <v>109</v>
       </c>
@@ -7031,7 +7031,7 @@
       <c r="A12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="12" t="s">
         <v>110</v>
       </c>
@@ -7056,7 +7056,7 @@
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="25"/>
       <c r="F13" s="12" t="s">
         <v>111</v>
       </c>
@@ -7080,7 +7080,7 @@
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="18"/>
+      <c r="E14" s="25"/>
       <c r="F14" s="12" t="s">
         <v>112</v>
       </c>
@@ -7104,42 +7104,42 @@
       <c r="A15" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="18"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E17" s="18"/>
+      <c r="E17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="B18" s="25"/>
+      <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="18"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="18"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="B21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -7148,22 +7148,22 @@
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="18"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="18"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E24" s="18"/>
+      <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E25" s="18"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -7172,139 +7172,139 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E26" s="18"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E28" s="18"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E29" s="18"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E30" s="18"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E31" s="18"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E32" s="18"/>
+      <c r="E32" s="25"/>
     </row>
     <row r="33" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E33" s="18"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E34" s="18"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E35" s="18"/>
+      <c r="E35" s="25"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E36" s="18"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E37" s="18"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E38" s="18"/>
+      <c r="E38" s="25"/>
     </row>
     <row r="39" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E39" s="18"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E40" s="18"/>
+      <c r="E40" s="25"/>
     </row>
     <row r="41" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E41" s="18"/>
+      <c r="E41" s="25"/>
     </row>
     <row r="42" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E42" s="18"/>
+      <c r="E42" s="25"/>
     </row>
     <row r="43" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E43" s="18"/>
+      <c r="E43" s="25"/>
     </row>
     <row r="44" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E44" s="18"/>
+      <c r="E44" s="25"/>
     </row>
     <row r="45" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E45" s="18"/>
+      <c r="E45" s="25"/>
     </row>
     <row r="46" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E46" s="18"/>
+      <c r="E46" s="25"/>
     </row>
     <row r="47" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E47" s="18"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" spans="5:9" x14ac:dyDescent="0.2">
-      <c r="E48" s="18"/>
+      <c r="E48" s="25"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="18"/>
+      <c r="E49" s="25"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="18"/>
+      <c r="E50" s="25"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="18"/>
+      <c r="E51" s="25"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="18"/>
+      <c r="E52" s="25"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="18"/>
+      <c r="E53" s="25"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="18"/>
+      <c r="E54" s="25"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="18"/>
+      <c r="E55" s="25"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="18"/>
+      <c r="E56" s="25"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="18"/>
+      <c r="E57" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7347,6 +7347,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
@@ -7355,15 +7364,6 @@
     <TaxCatchAll xmlns="be71ce3a-ef61-410b-aae3-59cf01e8169d" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7568,6 +7568,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31EB17D4-6620-41BA-83C9-0358F4652F7C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23DA2851-01F3-47E7-96BF-9362FC37866B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -7580,14 +7588,6 @@
     <ds:schemaRef ds:uri="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31EB17D4-6620-41BA-83C9-0358F4652F7C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Enhance 2025 Annual Report on Drug-Related Mortality by adding treemap visualizations and updating figure generation scripts. Key changes include: - Introduced a new treemap figure type for visualizing substance classification in overdose deaths. - Updated the figure builder to support treemap creation with consistent styling. - Modified the registry renderer to handle treemap figures and adjusted workbook loader for new figure type recognition. - Added new tables and figures in the data chapter to reflect updated overdose statistics and trends.
</commit_message>
<xml_diff>
--- a/data/raw/workbook.xlsx
+++ b/data/raw/workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Work Drive/GitHub/2025 Annual Report on Drug Related Mortality/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC88794-F1E0-264E-A188-EA72C858A792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0491F838-6234-0640-A021-D7C8B1C24151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -5436,7 +5436,7 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="E11" s="25"/>
       <c r="G11" s="2"/>
@@ -7356,17 +7356,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="be71ce3a-ef61-410b-aae3-59cf01e8169d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E06BBCF48891B4AA000B842D02367CE" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe6ea1b7fa6cedb1acda08ea4d5bc607">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="70db5d92-cf7a-41c9-a808-9efa4eb812f2" xmlns:ns3="be71ce3a-ef61-410b-aae3-59cf01e8169d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c75d4e196960d1be8fe94f46d8363ec" ns2:_="" ns3:_="">
     <xsd:import namespace="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
@@ -7567,6 +7556,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="be71ce3a-ef61-410b-aae3-59cf01e8169d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31EB17D4-6620-41BA-83C9-0358F4652F7C}">
   <ds:schemaRefs>
@@ -7576,23 +7576,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23DA2851-01F3-47E7-96BF-9362FC37866B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="be71ce3a-ef61-410b-aae3-59cf01e8169d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF5969E4-39DE-4C93-A7E1-5338058A9C0D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7609,4 +7592,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23DA2851-01F3-47E7-96BF-9362FC37866B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="be71ce3a-ef61-410b-aae3-59cf01e8169d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Pull workbook sources and notes into the data chapter: include tables under figures, add top 10 substances table
</commit_message>
<xml_diff>
--- a/data/raw/workbook.xlsx
+++ b/data/raw/workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Work Drive/GitHub/2025 Annual Report on Drug Related Mortality/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0491F838-6234-0640-A021-D7C8B1C24151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28E6663-2FD7-434A-8239-F792DC430296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="Drugs Present Time OD Death" sheetId="13" r:id="rId9"/>
     <sheet name="Drugs in Tox Screening 24" sheetId="14" r:id="rId10"/>
     <sheet name="OD Deaths OpioidStim 21-24" sheetId="15" r:id="rId11"/>
-    <sheet name="Template2 (2)" sheetId="16" r:id="rId12"/>
+    <sheet name="Top 10 Substances" sheetId="16" r:id="rId12"/>
     <sheet name="Sheet2" sheetId="8" r:id="rId13"/>
     <sheet name="Template2" sheetId="5" r:id="rId14"/>
   </sheets>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="156">
   <si>
     <t>Activate/Deactivate</t>
   </si>
@@ -1453,6 +1453,15 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
       <c r="E11" s="22" t="s">
         <v>152</v>
       </c>
@@ -2587,13 +2596,13 @@
         <v>55</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>22</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>22</v>
@@ -7356,6 +7365,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="be71ce3a-ef61-410b-aae3-59cf01e8169d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E06BBCF48891B4AA000B842D02367CE" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe6ea1b7fa6cedb1acda08ea4d5bc607">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="70db5d92-cf7a-41c9-a808-9efa4eb812f2" xmlns:ns3="be71ce3a-ef61-410b-aae3-59cf01e8169d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c75d4e196960d1be8fe94f46d8363ec" ns2:_="" ns3:_="">
     <xsd:import namespace="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
@@ -7556,17 +7576,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="be71ce3a-ef61-410b-aae3-59cf01e8169d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31EB17D4-6620-41BA-83C9-0358F4652F7C}">
   <ds:schemaRefs>
@@ -7576,6 +7585,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23DA2851-01F3-47E7-96BF-9362FC37866B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="be71ce3a-ef61-410b-aae3-59cf01e8169d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF5969E4-39DE-4C93-A7E1-5338058A9C0D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7592,21 +7618,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23DA2851-01F3-47E7-96BF-9362FC37866B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="be71ce3a-ef61-410b-aae3-59cf01e8169d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Point data chapter treemap at fig-8/tbl-8, update caption and 2025 substance counts
</commit_message>
<xml_diff>
--- a/data/raw/workbook.xlsx
+++ b/data/raw/workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Work Drive/GitHub/2025 Annual Report on Drug Related Mortality/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28E6663-2FD7-434A-8239-F792DC430296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEAB843D-DE0C-8A49-9A70-ECFCD061C16F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,9 @@
     <sheet name="OD Death Quarter 21-24" sheetId="9" r:id="rId5"/>
     <sheet name="OD Deaths Pop 21-24" sheetId="10" r:id="rId6"/>
     <sheet name="OD Deaths Sex 21-24" sheetId="11" r:id="rId7"/>
-    <sheet name="Overdose Deaths Age Group 21-24" sheetId="12" r:id="rId8"/>
+    <sheet name="Deaths by Substance Class" sheetId="14" r:id="rId8"/>
     <sheet name="Drugs Present Time OD Death" sheetId="13" r:id="rId9"/>
-    <sheet name="Drugs in Tox Screening 24" sheetId="14" r:id="rId10"/>
+    <sheet name="Overdose Deaths Age Group 21-24" sheetId="12" r:id="rId10"/>
     <sheet name="OD Deaths OpioidStim 21-24" sheetId="15" r:id="rId11"/>
     <sheet name="Top 10 Substances" sheetId="16" r:id="rId12"/>
     <sheet name="Sheet2" sheetId="8" r:id="rId13"/>
@@ -276,9 +276,6 @@
     <t>Type of Drugs Present at Time of Overdose Death, 2022-2024</t>
   </si>
   <si>
-    <t>Share of Occurrences of Select Drugs in Toxicology Screenings, 2024</t>
-  </si>
-  <si>
     <t>Percent of Overdose Deaths by Opioid and Stimulant Involvement, 2021-2024</t>
   </si>
   <si>
@@ -391,9 +388,6 @@
   </si>
   <si>
     <t>Drug</t>
-  </si>
-  <si>
-    <t>Occurrences</t>
   </si>
   <si>
     <t>All Opioids</t>
@@ -515,6 +509,12 @@
   </si>
   <si>
     <t>Note: The drugs in this table have not been categorized into broader classifications and represent the true, standalone occurrences of each specific substance. While these substances were present in toxicology findings at the time of death, they may not have been the direct cause of death. Furthermore, additional drugs or compounds may have been present; however, this dataset is strictly limited to these ten drugs. The list is not mutually exclusive, as a single multi-substance fatality can contribute to the counts of multiple drugs. For this reason, the cumulative counts do not equal the 67 overall deaths recorded in 2025. For reference, there were 78 deaths in 2024.</t>
+  </si>
+  <si>
+    <t>Deaths by Substance Class, 2025</t>
+  </si>
+  <si>
+    <t>Deaths</t>
   </si>
 </sst>
 </file>
@@ -1298,13 +1298,13 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -1324,10 +1324,10 @@
         <v>69</v>
       </c>
       <c r="F3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -1341,10 +1341,10 @@
         <v>70</v>
       </c>
       <c r="F4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -1358,10 +1358,10 @@
         <v>71</v>
       </c>
       <c r="F5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1375,10 +1375,10 @@
         <v>72</v>
       </c>
       <c r="F6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1392,10 +1392,10 @@
         <v>73</v>
       </c>
       <c r="F7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -1412,10 +1412,10 @@
         <v>75</v>
       </c>
       <c r="F8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -1426,13 +1426,13 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>76</v>
+        <v>154</v>
       </c>
       <c r="F9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -1443,13 +1443,13 @@
         <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
@@ -1463,13 +1463,13 @@
         <v>11</v>
       </c>
       <c r="E11" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="F11" t="s">
+        <v>151</v>
+      </c>
+      <c r="G11" t="s">
         <v>152</v>
-      </c>
-      <c r="F11" t="s">
-        <v>153</v>
-      </c>
-      <c r="G11" t="s">
-        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1479,7 +1479,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F3602D-0521-4D89-8267-3EDAFA503D89}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A70B9CED-0239-4594-A45D-902F01FA8F74}">
   <dimension ref="A1:Q57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1487,8 +1487,8 @@
     <col min="2" max="2" width="22.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.6640625" customWidth="1"/>
     <col min="6" max="6" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.83203125" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.83203125" bestFit="1" customWidth="1"/>
@@ -1503,7 +1503,7 @@
         <v>37</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="B3" t="str">
         <f>IF($B$1="","",_xlfn.XLOOKUP($B$1,Master!$E$2:$E$321,Master!$F$2:$F$321,""))</f>
-        <v>tbl-8</v>
+        <v>tbl-6</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -1542,20 +1542,24 @@
       </c>
       <c r="B4" t="str">
         <f>IF($B$1="","",_xlfn.XLOOKUP($B$1,Master!$E$2:$E$321,Master!$G$2:$G$321,""))</f>
-        <v>fig-8</v>
+        <v>fig-6</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
+        <v>22</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
@@ -1564,7 +1568,7 @@
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
     </row>
-    <row r="5" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
@@ -1572,14 +1576,20 @@
       <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>115</v>
+      <c r="F5" t="s">
+        <v>98</v>
+      </c>
+      <c r="G5">
+        <v>2021</v>
+      </c>
+      <c r="H5">
+        <v>2022</v>
+      </c>
+      <c r="I5">
+        <v>2023</v>
+      </c>
+      <c r="J5">
+        <v>2024</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1590,17 +1600,21 @@
         <v>0</v>
       </c>
       <c r="E6" s="25"/>
-      <c r="F6" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="H6" s="9">
-        <v>48</v>
-      </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="F6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G6" s="8">
+        <v>14.7</v>
+      </c>
+      <c r="H6" s="8">
+        <v>10.9</v>
+      </c>
+      <c r="I6" s="8">
+        <v>10.9</v>
+      </c>
+      <c r="J6" s="8">
+        <v>9.3000000000000007</v>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -1609,97 +1623,97 @@
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E7" s="25"/>
-      <c r="F7" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="H7" s="9">
-        <v>7</v>
-      </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="F7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" s="8">
+        <v>90.1</v>
+      </c>
+      <c r="H7" s="8">
+        <v>71.8</v>
+      </c>
+      <c r="I7" s="8">
+        <v>66.3</v>
+      </c>
+      <c r="J7" s="8">
+        <v>40.200000000000003</v>
+      </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="E8" s="25"/>
-      <c r="F8" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="H8" s="9">
-        <v>4</v>
-      </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="F8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G8" s="8">
+        <v>60</v>
+      </c>
+      <c r="H8" s="8">
+        <v>59.2</v>
+      </c>
+      <c r="I8" s="8">
+        <v>58.2</v>
+      </c>
+      <c r="J8" s="8">
+        <v>33</v>
+      </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
       <c r="B9" s="25"/>
       <c r="E9" s="25"/>
-      <c r="F9" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="H9" s="9">
-        <v>3</v>
-      </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+      <c r="F9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G9" s="8">
+        <v>35.5</v>
+      </c>
+      <c r="H9" s="8">
+        <v>49.1</v>
+      </c>
+      <c r="I9" s="8">
+        <v>28.3</v>
+      </c>
+      <c r="J9" s="8">
+        <v>21</v>
+      </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>53</v>
       </c>
       <c r="E10" s="25"/>
-      <c r="F10" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="H10" s="9">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
+      <c r="B11" t="s">
+        <v>80</v>
+      </c>
       <c r="E11" s="25"/>
-      <c r="F11" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="H11" s="9">
-        <v>7</v>
-      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -1707,54 +1721,33 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>42</v>
       </c>
       <c r="E12" s="25"/>
-      <c r="F12" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="H12" s="9">
-        <v>20</v>
-      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>43</v>
       </c>
       <c r="E13" s="25"/>
-      <c r="F13" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H13" s="9">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
       <c r="E14" s="25"/>
-      <c r="F14" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="H14" s="9">
-        <v>10</v>
-      </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -1789,7 +1782,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -1809,12 +1802,12 @@
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="342" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="17" t="s">
-        <v>144</v>
+      <c r="B22" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="E22" s="25"/>
       <c r="F22" s="2"/>
@@ -1985,13 +1978,13 @@
     <mergeCell ref="A27:B27"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10" xr:uid="{95B96CA0-6EA9-4F6C-B072-545CD855DA44}">
-      <formula1>"Line,Clustered Bar,Stacked Bar,Bar,Horizontal Stacked Bar,Treemap"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10" xr:uid="{FF4DF22E-1925-4A03-BB91-CCB2BF51D646}">
+      <formula1>"Line,Clustered Bar,Stacked Bar,Bar,Horizontal Stacked Bar"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{395CA644-C5B6-481A-875B-4254450F1887}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{4B200F09-3F53-44BB-859C-79A7DACF4BD5}">
       <formula1>"Table,Figure,Both"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6 B15:B16" xr:uid="{AF3D6EF1-DAD3-4C31-8D4A-6635E14D12C7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6 B15:B16" xr:uid="{7E5E9F2E-7BB9-4B8C-A0C7-AC4197F9957A}">
       <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1999,7 +1992,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DF0F3E81-D988-4AF9-BB13-972A146C0BC1}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{07FC8B81-2F27-4ECF-84AC-462B5AE912D2}">
           <x14:formula1>
             <xm:f>Master!$E$2:$E$10</xm:f>
           </x14:formula1>
@@ -2036,7 +2029,7 @@
         <v>37</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -2131,7 +2124,7 @@
       </c>
       <c r="E6" s="25"/>
       <c r="F6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G6" s="8">
         <v>34.6</v>
@@ -2154,7 +2147,7 @@
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E7" s="25"/>
       <c r="F7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G7" s="8">
         <v>34.6</v>
@@ -2177,7 +2170,7 @@
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="E8" s="25"/>
       <c r="F8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G8" s="8">
         <v>20.5</v>
@@ -2204,7 +2197,7 @@
       <c r="B9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G9" s="8">
         <v>10.3</v>
@@ -2229,7 +2222,7 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E10" s="25"/>
       <c r="G10" s="2"/>
@@ -2306,7 +2299,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -2550,7 +2543,7 @@
         <v>37</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -2624,7 +2617,7 @@
         <v>54</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G5" s="38">
         <v>2025</v>
@@ -2665,7 +2658,7 @@
     <row r="7" spans="1:17" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E7" s="25"/>
       <c r="F7" s="19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G7" s="20">
         <v>40</v>
@@ -2688,7 +2681,7 @@
     <row r="8" spans="1:17" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E8" s="25"/>
       <c r="F8" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G8" s="20">
         <v>36</v>
@@ -2715,7 +2708,7 @@
       <c r="B9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="19" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G9" s="20">
         <v>14</v>
@@ -2741,7 +2734,7 @@
       </c>
       <c r="E10" s="25"/>
       <c r="F10" s="19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G10" s="20">
         <v>8</v>
@@ -2762,7 +2755,7 @@
       </c>
       <c r="E11" s="25"/>
       <c r="F11" s="19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G11" s="20">
         <v>7</v>
@@ -2787,7 +2780,7 @@
       </c>
       <c r="E12" s="25"/>
       <c r="F12" s="19" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G12" s="20">
         <v>5</v>
@@ -2810,7 +2803,7 @@
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="19" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G13" s="20">
         <v>5</v>
@@ -2831,7 +2824,7 @@
       </c>
       <c r="E14" s="25"/>
       <c r="F14" s="19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G14" s="20">
         <v>4</v>
@@ -2852,7 +2845,7 @@
       </c>
       <c r="E15" s="25"/>
       <c r="F15" s="19" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="G15" s="20">
         <v>4</v>
@@ -2873,7 +2866,7 @@
       </c>
       <c r="E16" s="25"/>
       <c r="F16" s="19" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="G16" s="20">
         <v>4</v>
@@ -2903,7 +2896,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -2928,7 +2921,7 @@
         <v>48</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E22" s="25"/>
       <c r="F22" s="2"/>
@@ -3817,7 +3810,7 @@
         <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G5">
         <v>2024</v>
@@ -3935,7 +3928,7 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E11" s="25"/>
       <c r="F11" t="s">
@@ -4045,7 +4038,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -4345,7 +4338,7 @@
         <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" t="s">
         <v>1</v>
@@ -4434,7 +4427,7 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E10" s="25"/>
       <c r="G10" s="2"/>
@@ -4444,7 +4437,7 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E11" s="25"/>
       <c r="G11" s="2"/>
@@ -4829,19 +4822,19 @@
         <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" t="s">
         <v>83</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>84</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>85</v>
-      </c>
-      <c r="J5" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -4961,7 +4954,7 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E11" s="25"/>
       <c r="G11" s="2"/>
@@ -5031,7 +5024,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -5370,7 +5363,7 @@
       </c>
       <c r="E6" s="25"/>
       <c r="F6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G6" s="2">
         <v>35.9</v>
@@ -5445,7 +5438,7 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E11" s="25"/>
       <c r="G11" s="2"/>
@@ -5515,7 +5508,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -5833,7 +5826,7 @@
         <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G5">
         <v>2021</v>
@@ -5857,7 +5850,7 @@
       </c>
       <c r="E6" s="25"/>
       <c r="F6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G6" s="2">
         <v>46.9</v>
@@ -5880,7 +5873,7 @@
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E7" s="25"/>
       <c r="F7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G7" s="2">
         <v>24.3</v>
@@ -5943,7 +5936,7 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E11" s="25"/>
       <c r="G11" s="2"/>
@@ -6016,7 +6009,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -6041,7 +6034,7 @@
         <v>48</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E22" s="25"/>
       <c r="F22" s="2"/>
@@ -6239,7 +6232,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A70B9CED-0239-4594-A45D-902F01FA8F74}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F3602D-0521-4D89-8267-3EDAFA503D89}">
   <dimension ref="A1:Q57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -6247,8 +6240,8 @@
     <col min="2" max="2" width="22.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.6640625" customWidth="1"/>
     <col min="6" max="6" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.83203125" customWidth="1"/>
     <col min="9" max="9" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.83203125" bestFit="1" customWidth="1"/>
@@ -6263,7 +6256,7 @@
         <v>37</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>73</v>
+        <v>154</v>
       </c>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -6293,7 +6286,7 @@
       </c>
       <c r="B3" t="str">
         <f>IF($B$1="","",_xlfn.XLOOKUP($B$1,Master!$E$2:$E$321,Master!$F$2:$F$321,""))</f>
-        <v>tbl-6</v>
+        <v>tbl-8</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -6302,24 +6295,20 @@
       </c>
       <c r="B4" t="str">
         <f>IF($B$1="","",_xlfn.XLOOKUP($B$1,Master!$E$2:$E$321,Master!$G$2:$G$321,""))</f>
-        <v>fig-6</v>
+        <v>fig-8</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>22</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
@@ -6328,7 +6317,7 @@
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="26" t="s">
         <v>38</v>
       </c>
@@ -6336,20 +6325,14 @@
       <c r="E5" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="F5" t="s">
-        <v>99</v>
-      </c>
-      <c r="G5">
-        <v>2021</v>
-      </c>
-      <c r="H5">
-        <v>2022</v>
-      </c>
-      <c r="I5">
-        <v>2023</v>
-      </c>
-      <c r="J5">
-        <v>2024</v>
+      <c r="F5" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -6360,21 +6343,17 @@
         <v>0</v>
       </c>
       <c r="E6" s="25"/>
-      <c r="F6" t="s">
-        <v>95</v>
-      </c>
-      <c r="G6" s="8">
-        <v>14.7</v>
-      </c>
-      <c r="H6" s="8">
-        <v>10.9</v>
-      </c>
-      <c r="I6" s="8">
-        <v>10.9</v>
-      </c>
-      <c r="J6" s="8">
-        <v>9.3000000000000007</v>
-      </c>
+      <c r="F6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H6" s="9">
+        <v>36</v>
+      </c>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -6383,97 +6362,97 @@
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E7" s="25"/>
-      <c r="F7" t="s">
-        <v>96</v>
-      </c>
-      <c r="G7" s="8">
-        <v>90.1</v>
-      </c>
-      <c r="H7" s="8">
-        <v>71.8</v>
-      </c>
-      <c r="I7" s="8">
-        <v>66.3</v>
-      </c>
-      <c r="J7" s="8">
-        <v>40.200000000000003</v>
-      </c>
+      <c r="F7" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="H7" s="9">
+        <v>5</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="E8" s="25"/>
-      <c r="F8" t="s">
-        <v>97</v>
-      </c>
-      <c r="G8" s="8">
-        <v>60</v>
-      </c>
-      <c r="H8" s="8">
-        <v>59.2</v>
-      </c>
-      <c r="I8" s="8">
-        <v>58.2</v>
-      </c>
-      <c r="J8" s="8">
-        <v>33</v>
-      </c>
+      <c r="F8" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="H8" s="9">
+        <v>7</v>
+      </c>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
         <v>40</v>
       </c>
       <c r="B9" s="25"/>
       <c r="E9" s="25"/>
-      <c r="F9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G9" s="8">
-        <v>35.5</v>
-      </c>
-      <c r="H9" s="8">
-        <v>49.1</v>
-      </c>
-      <c r="I9" s="8">
-        <v>28.3</v>
-      </c>
-      <c r="J9" s="8">
-        <v>21</v>
-      </c>
+      <c r="F9" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="H9" s="9">
+        <v>7</v>
+      </c>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="E10" s="25"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="F10" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" s="9">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" t="s">
-        <v>81</v>
-      </c>
       <c r="E11" s="25"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="F11" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H11" s="9">
+        <v>2</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -6481,33 +6460,54 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>42</v>
       </c>
       <c r="E12" s="25"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
+      <c r="F12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H12" s="9">
+        <v>14</v>
+      </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>43</v>
       </c>
       <c r="E13" s="25"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="F13" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="H13" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="B14" t="s">
-        <v>27</v>
-      </c>
       <c r="E14" s="25"/>
+      <c r="F14" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H14" s="9">
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -6542,7 +6542,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E19" s="25"/>
     </row>
@@ -6562,12 +6562,12 @@
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="342" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>94</v>
+      <c r="B22" s="17" t="s">
+        <v>142</v>
       </c>
       <c r="E22" s="25"/>
       <c r="F22" s="2"/>
@@ -6738,13 +6738,13 @@
     <mergeCell ref="A27:B27"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10" xr:uid="{FF4DF22E-1925-4A03-BB91-CCB2BF51D646}">
-      <formula1>"Line,Clustered Bar,Stacked Bar,Bar,Horizontal Stacked Bar"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10" xr:uid="{95B96CA0-6EA9-4F6C-B072-545CD855DA44}">
+      <formula1>"Line,Clustered Bar,Stacked Bar,Bar,Horizontal Stacked Bar,Treemap"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{4B200F09-3F53-44BB-859C-79A7DACF4BD5}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{395CA644-C5B6-481A-875B-4254450F1887}">
       <formula1>"Table,Figure,Both"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6 B15:B16" xr:uid="{7E5E9F2E-7BB9-4B8C-A0C7-AC4197F9957A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6 B15:B16" xr:uid="{AF3D6EF1-DAD3-4C31-8D4A-6635E14D12C7}">
       <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6752,7 +6752,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{07FC8B81-2F27-4ECF-84AC-462B5AE912D2}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DF0F3E81-D988-4AF9-BB13-972A146C0BC1}">
           <x14:formula1>
             <xm:f>Master!$E$2:$E$10</xm:f>
           </x14:formula1>
@@ -6865,15 +6865,15 @@
         <v>54</v>
       </c>
       <c r="F5" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="31" t="s">
         <v>100</v>
-      </c>
-      <c r="G5" s="31" t="s">
-        <v>101</v>
       </c>
       <c r="H5" s="32"/>
       <c r="I5" s="33"/>
       <c r="J5" s="34" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K5" s="35"/>
     </row>
@@ -6896,10 +6896,10 @@
         <v>2024</v>
       </c>
       <c r="J6" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="K6" s="10" t="s">
         <v>103</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>104</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -6909,7 +6909,7 @@
     <row r="7" spans="1:17" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E7" s="25"/>
       <c r="F7" s="12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G7" s="13">
         <v>112</v>
@@ -6934,7 +6934,7 @@
     <row r="8" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E8" s="25"/>
       <c r="F8" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G8" s="13">
         <v>35</v>
@@ -6963,7 +6963,7 @@
       <c r="B9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G9" s="13">
         <v>18</v>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="E10" s="25"/>
       <c r="F10" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G10" s="13">
         <v>27</v>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="E11" s="25"/>
       <c r="F11" s="12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G11" s="13">
         <v>18</v>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="E12" s="25"/>
       <c r="F12" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G12" s="13">
         <v>2</v>
@@ -7067,7 +7067,7 @@
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G13" s="13">
         <v>22</v>
@@ -7091,7 +7091,7 @@
       </c>
       <c r="E14" s="25"/>
       <c r="F14" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G14" s="13">
         <v>23</v>
@@ -7356,26 +7356,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="be71ce3a-ef61-410b-aae3-59cf01e8169d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E06BBCF48891B4AA000B842D02367CE" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe6ea1b7fa6cedb1acda08ea4d5bc607">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="70db5d92-cf7a-41c9-a808-9efa4eb812f2" xmlns:ns3="be71ce3a-ef61-410b-aae3-59cf01e8169d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c75d4e196960d1be8fe94f46d8363ec" ns2:_="" ns3:_="">
     <xsd:import namespace="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
@@ -7576,10 +7556,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="be71ce3a-ef61-410b-aae3-59cf01e8169d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31EB17D4-6620-41BA-83C9-0358F4652F7C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF5969E4-39DE-4C93-A7E1-5338058A9C0D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
+    <ds:schemaRef ds:uri="be71ce3a-ef61-410b-aae3-59cf01e8169d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7602,20 +7613,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF5969E4-39DE-4C93-A7E1-5338058A9C0D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31EB17D4-6620-41BA-83C9-0358F4652F7C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
-    <ds:schemaRef ds:uri="be71ce3a-ef61-410b-aae3-59cf01e8169d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>